<commit_message>
Added some timetable to Year 2
</commit_message>
<xml_diff>
--- a/Progress-Trackers/Year-2.xlsx
+++ b/Progress-Trackers/Year-2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Documents\GitHub\Module-Summaries\Progress-Trackers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D64D97-62D5-457B-A24B-8B7C156E20DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF15EACE-9641-4633-B443-2D0050D4522D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="48">
   <si>
     <t>Lecture</t>
   </si>
@@ -80,9 +80,6 @@
     <t>1x2hr</t>
   </si>
   <si>
-    <t>Practical</t>
-  </si>
-  <si>
     <t>Assessment:</t>
   </si>
   <si>
@@ -191,9 +188,6 @@
     <t>Location</t>
   </si>
   <si>
-    <t>Room</t>
-  </si>
-  <si>
     <t>Today's Timetable</t>
   </si>
   <si>
@@ -201,6 +195,15 @@
   </si>
   <si>
     <t>Code</t>
+  </si>
+  <si>
+    <t>CLC202</t>
+  </si>
+  <si>
+    <t>W103</t>
+  </si>
+  <si>
+    <t>TLC033</t>
   </si>
 </sst>
 </file>
@@ -388,7 +391,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -428,22 +431,11 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -454,19 +446,23 @@
     <xf numFmtId="2" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="20" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="20" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="56">
+  <dxfs count="13">
     <dxf>
       <font>
         <color rgb="FFCCFF99"/>
@@ -582,385 +578,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFCCFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF99"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC66"/>
-        </patternFill>
-      </fill>
-      <border>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFF99"/>
-        </patternFill>
-      </fill>
-      <border>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.14996795556505021"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFF99"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC66"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-      <border>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF99"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.14996795556505021"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC66"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-      <border>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF99"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="2" tint="-0.749961851863155"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC66"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-      <border>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC66"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-      <border>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF99"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-      <border>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC66"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF99"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF7C80"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFCCFF66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFCC66"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC66"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1267,7 +884,7 @@
     <col min="1" max="1" width="8.7265625" style="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="12" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="14.6328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6328125" style="24" customWidth="1"/>
+    <col min="6" max="6" width="14.6328125" style="21" customWidth="1"/>
     <col min="7" max="11" width="14.6328125" style="1" customWidth="1"/>
     <col min="12" max="12" width="3.1796875" style="1" customWidth="1"/>
     <col min="13" max="16384" width="8.7265625" style="1"/>
@@ -1279,7 +896,7 @@
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
-      <c r="F2" s="25"/>
+      <c r="F2" s="22"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
@@ -1319,20 +936,20 @@
       <c r="L3" s="8"/>
     </row>
     <row r="4" spans="2:12" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="28" t="s">
-        <v>34</v>
+      <c r="B4" s="24" t="s">
+        <v>33</v>
       </c>
       <c r="C4" s="19" t="str">
         <f>Calculator!D1</f>
-        <v>Lecture Part 1</v>
+        <v>None</v>
       </c>
       <c r="D4" s="19" t="str">
         <f>Calculator!E1</f>
-        <v>Lecture Part 2</v>
+        <v>None</v>
       </c>
       <c r="E4" s="19" t="str">
         <f>Calculator!F1</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="F4" s="19" t="str">
         <f>Calculator!G1</f>
@@ -1352,33 +969,33 @@
       </c>
       <c r="J4" s="19" t="str">
         <f>Calculator!K1</f>
-        <v>Practical Part 1</v>
+        <v>None</v>
       </c>
       <c r="K4" s="19" t="str">
         <f>Calculator!L1</f>
-        <v>Practical Part 2</v>
+        <v>None</v>
       </c>
       <c r="L4" s="8"/>
     </row>
     <row r="5" spans="2:12" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="28" t="s">
-        <v>38</v>
+      <c r="B5" s="24" t="s">
+        <v>37</v>
       </c>
       <c r="C5" s="19" t="str">
         <f>Calculator!D2</f>
-        <v>Practical Part 1</v>
+        <v>Lecture</v>
       </c>
       <c r="D5" s="19" t="str">
         <f>Calculator!E2</f>
-        <v>Practical Part 2</v>
+        <v>Lecture</v>
       </c>
       <c r="E5" s="19" t="str">
         <f>Calculator!F2</f>
-        <v>Practical Part 1</v>
+        <v>None</v>
       </c>
       <c r="F5" s="19" t="str">
         <f>Calculator!G2</f>
-        <v>Practical Part 2</v>
+        <v>None</v>
       </c>
       <c r="G5" s="19" t="str">
         <f>Calculator!H2</f>
@@ -1386,15 +1003,15 @@
       </c>
       <c r="H5" s="19" t="str">
         <f>Calculator!I2</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="I5" s="19" t="str">
         <f>Calculator!J2</f>
-        <v>Practical Part 1</v>
+        <v>None</v>
       </c>
       <c r="J5" s="19" t="str">
         <f>Calculator!K2</f>
-        <v>Practical Part 2</v>
+        <v>None</v>
       </c>
       <c r="K5" s="19" t="str">
         <f>Calculator!L2</f>
@@ -1403,20 +1020,20 @@
       <c r="L5" s="8"/>
     </row>
     <row r="6" spans="2:12" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="28" t="s">
-        <v>39</v>
+      <c r="B6" s="24" t="s">
+        <v>38</v>
       </c>
       <c r="C6" s="19" t="str">
         <f>Calculator!D3</f>
-        <v>Workshop Part 1</v>
+        <v>None</v>
       </c>
       <c r="D6" s="19" t="str">
         <f>Calculator!E3</f>
-        <v>Workshop Part 2</v>
+        <v>None</v>
       </c>
       <c r="E6" s="19" t="str">
         <f>Calculator!F3</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="F6" s="19" t="str">
         <f>Calculator!G3</f>
@@ -1445,16 +1062,16 @@
       <c r="L6" s="8"/>
     </row>
     <row r="7" spans="2:12" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="28" t="s">
-        <v>40</v>
+      <c r="B7" s="24" t="s">
+        <v>39</v>
       </c>
       <c r="C7" s="19" t="str">
         <f>Calculator!D4</f>
-        <v>Lecture</v>
+        <v>Lecture Part 1</v>
       </c>
       <c r="D7" s="19" t="str">
         <f>Calculator!E4</f>
-        <v>None</v>
+        <v>Lecture Part 2</v>
       </c>
       <c r="E7" s="19" t="str">
         <f>Calculator!F4</f>
@@ -1466,11 +1083,11 @@
       </c>
       <c r="G7" s="19" t="str">
         <f>Calculator!H4</f>
-        <v>Lecture</v>
+        <v>None</v>
       </c>
       <c r="H7" s="19" t="str">
         <f>Calculator!I4</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="I7" s="19" t="str">
         <f>Calculator!J4</f>
@@ -1487,8 +1104,8 @@
       <c r="L7" s="8"/>
     </row>
     <row r="8" spans="2:12" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="28" t="s">
-        <v>41</v>
+      <c r="B8" s="24" t="s">
+        <v>40</v>
       </c>
       <c r="C8" s="19" t="str">
         <f>Calculator!D5</f>
@@ -1504,7 +1121,7 @@
       </c>
       <c r="F8" s="19" t="str">
         <f>Calculator!G5</f>
-        <v>Lecture</v>
+        <v>None</v>
       </c>
       <c r="G8" s="19" t="str">
         <f>Calculator!H5</f>
@@ -1512,11 +1129,11 @@
       </c>
       <c r="H8" s="19" t="str">
         <f>Calculator!I5</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="I8" s="19" t="str">
         <f>Calculator!J5</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="J8" s="19" t="str">
         <f>Calculator!K5</f>
@@ -1533,7 +1150,7 @@
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
-      <c r="F9" s="26"/>
+      <c r="F9" s="23"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
@@ -1543,71 +1160,89 @@
     </row>
     <row r="11" spans="2:12" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="B11" s="20" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E11" s="18" t="str">
         <f ca="1">TEXT(WEEKDAY(NOW()), "dddd")</f>
-        <v>Wednesday</v>
+        <v>Monday</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B13" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="30"/>
-      <c r="E13" s="29" t="s">
+      <c r="B13" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="31"/>
+      <c r="E13" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="F13" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="G13" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="H13" s="29" t="s">
-        <v>35</v>
+      <c r="G13" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="25" t="s">
+        <v>34</v>
       </c>
       <c r="I13" s="2"/>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="15" t="str" cm="1">
-        <f t="array" aca="1" ref="B14:C14" ca="1">_xlfn._xlws.FILTER(B28:C39, $F$28:$F$39=$E$11, "")</f>
-        <v>COMP2281</v>
+        <f t="array" aca="1" ref="B14:C15" ca="1">_xlfn._xlws.FILTER(B28:C39, $F$28:$F$39=$E$11, "")</f>
+        <v>COMP2221</v>
       </c>
       <c r="C14" s="15" t="str">
         <f ca="1"/>
-        <v>Software Engineering</v>
+        <v>Programming Paradigms</v>
       </c>
       <c r="D14" s="15"/>
       <c r="E14" s="15" t="str" cm="1">
-        <f t="array" aca="1" ref="E14" ca="1">_xlfn._xlws.FILTER(E28:E39, $F$28:$F$39=$E$11, "")</f>
-        <v>Workshop</v>
+        <f t="array" aca="1" ref="E14:E15" ca="1">_xlfn._xlws.FILTER(E28:E39, $F$28:$F$39=$E$11, "")</f>
+        <v>Lecture</v>
       </c>
       <c r="F14" s="17" cm="1">
-        <f t="array" aca="1" ref="F14:H14" ca="1">_xlfn._xlws.FILTER(G28:I39, $F$28:$F$39=$E$11, "")</f>
-        <v>9</v>
+        <f t="array" aca="1" ref="F14:H15" ca="1">_xlfn._xlws.FILTER(G28:I39, $F$28:$F$39=$E$11, "")</f>
+        <v>11</v>
       </c>
       <c r="G14" s="15" t="str">
         <f ca="1"/>
-        <v>Room</v>
+        <v>CLC202</v>
       </c>
       <c r="H14" s="15" t="str">
         <f ca="1"/>
-        <v>2 hours</v>
+        <v>1 hour</v>
       </c>
       <c r="I14" s="12"/>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
+      <c r="B15" s="15" t="str">
+        <f ca="1"/>
+        <v>COMP2271</v>
+      </c>
+      <c r="C15" s="15" t="str">
+        <f ca="1"/>
+        <v>Data Science</v>
+      </c>
       <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
+      <c r="E15" s="15" t="str">
+        <f ca="1"/>
+        <v>Lecture</v>
+      </c>
+      <c r="F15" s="17">
+        <f ca="1"/>
+        <v>12</v>
+      </c>
+      <c r="G15" s="15" t="str">
+        <f ca="1"/>
+        <v>W103</v>
+      </c>
+      <c r="H15" s="15" t="str">
+        <f ca="1"/>
+        <v>1 hour</v>
+      </c>
       <c r="I15" s="12"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.35">
@@ -1684,7 +1319,7 @@
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
       <c r="E23" s="12"/>
-      <c r="F23" s="32"/>
+      <c r="F23" s="27"/>
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
       <c r="I23" s="12"/>
@@ -1694,7 +1329,7 @@
     </row>
     <row r="25" spans="2:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="B25" s="20" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I25" s="12"/>
     </row>
@@ -1703,452 +1338,445 @@
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="28" t="s">
+        <v>32</v>
+      </c>
+      <c r="D27" s="28"/>
+      <c r="E27" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D27" s="21"/>
-      <c r="E27" s="2" t="s">
+      <c r="F27" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F27" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="H27" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B28" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C28" s="34" t="str">
-        <f>VLOOKUP(B28,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Networks and Systems</v>
-      </c>
-      <c r="D28" s="34"/>
+        <v>13</v>
+      </c>
+      <c r="C28" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B28, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Theory of Computation</v>
+      </c>
+      <c r="D28" s="29"/>
       <c r="E28" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="F28" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="G28" s="32">
-        <v>9</v>
+      <c r="F28" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="G28" s="27">
+        <v>10</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I28" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="J28" s="35" t="str">
+      <c r="J28" s="32" t="str">
         <f>_xlfn.CONCAT(F28, " ", G28)</f>
-        <v>Monday 9</v>
-      </c>
-      <c r="K28" s="1" t="str">
+        <v>Tuesday 10</v>
+      </c>
+      <c r="K28" s="18" t="str">
         <f>IF(I28="2 hours",_xlfn.CONCAT(F28," ",G28+1), "")</f>
-        <v>Monday 10</v>
+        <v/>
       </c>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B29" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C29" s="34" t="str">
-        <f>VLOOKUP(B29,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Networks and Systems</v>
-      </c>
-      <c r="D29" s="34"/>
+        <v>13</v>
+      </c>
+      <c r="C29" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B29, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Theory of Computation</v>
+      </c>
+      <c r="D29" s="29"/>
       <c r="E29" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="F29" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="G29" s="32">
-        <v>11</v>
+        <v>0</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G29" s="27">
+        <v>14</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I29" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="J29" s="35" t="str">
+      <c r="J29" s="32" t="str">
         <f t="shared" ref="J29:J39" si="0">_xlfn.CONCAT(F29, " ", G29)</f>
-        <v>Tuesday 11</v>
-      </c>
-      <c r="K29" s="1" t="str">
+        <v>Thursday 14</v>
+      </c>
+      <c r="K29" s="18" t="str">
         <f t="shared" ref="K29:K39" si="1">IF(I29="2 hours",_xlfn.CONCAT(F29," ",G29+1), "")</f>
-        <v>Tuesday 12</v>
+        <v/>
       </c>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B30" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C30" s="34" t="str">
-        <f>VLOOKUP(B30,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Programming Paradigms</v>
-      </c>
-      <c r="D30" s="34"/>
+        <v>1</v>
+      </c>
+      <c r="C30" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B30, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Networks and Systems</v>
+      </c>
+      <c r="D30" s="29"/>
       <c r="E30" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="F30" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="G30" s="32">
+      <c r="F30" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G30" s="27">
+        <v>9</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="I30" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="J30" s="32" t="str">
+        <f t="shared" si="0"/>
+        <v>Thursday 9</v>
+      </c>
+      <c r="K30" s="18" t="str">
+        <f t="shared" si="1"/>
+        <v>Thursday 10</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B31" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="H30" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I30" s="12" t="s">
+      <c r="C31" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B31, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Programming Paradigms</v>
+      </c>
+      <c r="D31" s="29"/>
+      <c r="E31" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="F31" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="G31" s="27">
+        <v>11</v>
+      </c>
+      <c r="H31" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="J31" s="32" t="str">
+        <f t="shared" si="0"/>
+        <v>Monday 11</v>
+      </c>
+      <c r="K31" s="18" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B32" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B32, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Programming Paradigms</v>
+      </c>
+      <c r="D32" s="29"/>
+      <c r="E32" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="G32" s="27">
+        <v>14</v>
+      </c>
+      <c r="H32" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="J32" s="32" t="str">
+        <f t="shared" si="0"/>
+        <v>Friday 14</v>
+      </c>
+      <c r="K32" s="18" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B33" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B33, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Artificial Intelligence</v>
+      </c>
+      <c r="D33" s="29"/>
+      <c r="E33" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="F33" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="J30" s="35" t="str">
+      <c r="G33" s="27">
+        <v>14</v>
+      </c>
+      <c r="H33" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="J33" s="32" t="str">
+        <f t="shared" si="0"/>
+        <v>Tuesday 14</v>
+      </c>
+      <c r="K33" s="18" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B34" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B34, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Artificial Intelligence</v>
+      </c>
+      <c r="D34" s="29"/>
+      <c r="E34" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="G34" s="27">
+        <v>15</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I34" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="J34" s="32" t="str">
+        <f t="shared" si="0"/>
+        <v>Friday 15</v>
+      </c>
+      <c r="K34" s="18" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B35" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B35, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Data Science</v>
+      </c>
+      <c r="D35" s="29"/>
+      <c r="E35" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="G35" s="27">
+        <v>12</v>
+      </c>
+      <c r="H35" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="J35" s="32" t="str">
+        <f t="shared" si="0"/>
+        <v>Monday 12</v>
+      </c>
+      <c r="K35" s="18" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B36" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B36, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Data Science</v>
+      </c>
+      <c r="D36" s="29"/>
+      <c r="E36" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="G36" s="27">
+        <v>10</v>
+      </c>
+      <c r="H36" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I36" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="J36" s="32" t="str">
         <f t="shared" si="0"/>
         <v>Friday 10</v>
       </c>
-      <c r="K30" s="1" t="str">
+      <c r="K36" s="18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B31" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C31" s="34" t="str">
-        <f>VLOOKUP(B31,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Programming Paradigms</v>
-      </c>
-      <c r="D31" s="34"/>
-      <c r="E31" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="F31" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="G31" s="32">
-        <v>16</v>
-      </c>
-      <c r="H31" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I31" s="12" t="s">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B37" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B37, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Software Engineering</v>
+      </c>
+      <c r="D37" s="29"/>
+      <c r="E37" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="G37" s="27">
+        <v>9</v>
+      </c>
+      <c r="H37" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="I37" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="J31" s="35" t="str">
+      <c r="J37" s="32" t="str">
         <f t="shared" si="0"/>
-        <v>Monday 16</v>
-      </c>
-      <c r="K31" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Monday 17</v>
-      </c>
-    </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B32" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C32" s="34" t="str">
-        <f>VLOOKUP(B32,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Theory of Computation</v>
-      </c>
-      <c r="D32" s="34"/>
-      <c r="E32" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="F32" s="33" t="s">
-        <v>40</v>
-      </c>
-      <c r="G32" s="32">
-        <v>9</v>
-      </c>
-      <c r="H32" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I32" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="J32" s="35" t="str">
-        <f t="shared" si="0"/>
-        <v>Thursday 9</v>
-      </c>
-      <c r="K32" s="1" t="str">
+        <v>Tuesday 9</v>
+      </c>
+      <c r="K37" s="18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B33" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C33" s="34" t="str">
-        <f>VLOOKUP(B33,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Theory of Computation</v>
-      </c>
-      <c r="D33" s="34"/>
-      <c r="E33" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="F33" s="33" t="s">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B38" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" s="29" t="str">
+        <f>_xlfn.XLOOKUP(B38, Calculator!$A$1:$A$6, Calculator!$B$1:$B$6, "Error", 0)</f>
+        <v>Software Engineering</v>
+      </c>
+      <c r="D38" s="29"/>
+      <c r="E38" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="F38" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G33" s="32">
-        <v>15</v>
-      </c>
-      <c r="H33" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I33" s="12" t="s">
+      <c r="G38" s="27">
+        <v>11</v>
+      </c>
+      <c r="H38" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="I38" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="J33" s="35" t="str">
+      <c r="J38" s="32" t="str">
         <f t="shared" si="0"/>
-        <v>Tuesday 15</v>
-      </c>
-      <c r="K33" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Tuesday 16</v>
-      </c>
-    </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B34" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C34" s="34" t="str">
-        <f>VLOOKUP(B34,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Artificial Intelligence</v>
-      </c>
-      <c r="D34" s="34"/>
-      <c r="E34" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="F34" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="G34" s="32">
-        <v>12</v>
-      </c>
-      <c r="H34" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I34" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="J34" s="35" t="str">
-        <f t="shared" si="0"/>
-        <v>Friday 12</v>
-      </c>
-      <c r="K34" s="1" t="str">
+        <v>Wednesday 11</v>
+      </c>
+      <c r="K38" s="18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B35" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C35" s="34" t="str">
-        <f>VLOOKUP(B35,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Artificial Intelligence</v>
-      </c>
-      <c r="D35" s="34"/>
-      <c r="E35" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="F35" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="G35" s="32">
-        <v>2</v>
-      </c>
-      <c r="H35" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I35" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="J35" s="35" t="str">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="C39" s="29"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="12"/>
+      <c r="J39" s="32" t="str">
         <f t="shared" si="0"/>
-        <v>Monday 2</v>
-      </c>
-      <c r="K35" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Monday 3</v>
-      </c>
-    </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B36" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="C36" s="34" t="str">
-        <f>VLOOKUP(B36,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Data Science</v>
-      </c>
-      <c r="D36" s="34"/>
-      <c r="E36" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="F36" s="33" t="s">
-        <v>40</v>
-      </c>
-      <c r="G36" s="32">
-        <v>13</v>
-      </c>
-      <c r="H36" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I36" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="J36" s="35" t="str">
-        <f t="shared" si="0"/>
-        <v>Thursday 13</v>
-      </c>
-      <c r="K36" s="1" t="str">
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="K39" s="18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B37" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="C37" s="34" t="str">
-        <f>VLOOKUP(B37,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Data Science</v>
-      </c>
-      <c r="D37" s="34"/>
-      <c r="E37" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="F37" s="33" t="s">
-        <v>38</v>
-      </c>
-      <c r="G37" s="32">
-        <v>9</v>
-      </c>
-      <c r="H37" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I37" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="J37" s="35" t="str">
-        <f t="shared" si="0"/>
-        <v>Tuesday 9</v>
-      </c>
-      <c r="K37" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Tuesday 10</v>
-      </c>
-    </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B38" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C38" s="34" t="str">
-        <f>VLOOKUP(B38,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Software Engineering</v>
-      </c>
-      <c r="D38" s="34"/>
-      <c r="E38" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="F38" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="G38" s="32">
-        <v>12</v>
-      </c>
-      <c r="H38" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I38" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="J38" s="35" t="str">
-        <f t="shared" si="0"/>
-        <v>Monday 12</v>
-      </c>
-      <c r="K38" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B39" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C39" s="34" t="str">
-        <f>VLOOKUP(B39,Calculator!$A$1:$B$6, 2, FALSE)</f>
-        <v>Software Engineering</v>
-      </c>
-      <c r="D39" s="34"/>
-      <c r="E39" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="F39" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="G39" s="32">
-        <v>9</v>
-      </c>
-      <c r="H39" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="I39" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="J39" s="35" t="str">
-        <f t="shared" si="0"/>
-        <v>Wednesday 9</v>
-      </c>
-      <c r="K39" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Wednesday 10</v>
-      </c>
+    <row r="40" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="J40" s="18"/>
+      <c r="K40" s="18"/>
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
+      <c r="C41" s="30"/>
+      <c r="D41" s="30"/>
+      <c r="J41" s="18"/>
+      <c r="K41" s="18"/>
     </row>
     <row r="42" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
+      <c r="C42" s="30"/>
+      <c r="D42" s="30"/>
     </row>
     <row r="54" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F54" s="23"/>
+      <c r="F54" s="1"/>
     </row>
     <row r="55" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F55" s="23"/>
+      <c r="F55" s="1"/>
     </row>
     <row r="56" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F56" s="23"/>
+      <c r="F56" s="1"/>
     </row>
     <row r="57" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F57" s="23"/>
+      <c r="F57" s="1"/>
     </row>
     <row r="58" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F58" s="23"/>
+      <c r="F58" s="1"/>
     </row>
     <row r="59" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F59" s="23"/>
+      <c r="F59" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C13:D13"/>
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="C39:D39"/>
@@ -2162,9 +1790,6 @@
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C13:D13"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="C4:K8">
@@ -2238,15 +1863,15 @@
       </c>
       <c r="D1" t="str" cm="1">
         <f t="array" ref="D1">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(E1 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Lecture Part 1</v>
+        <v>None</v>
       </c>
       <c r="E1" t="str" cm="1">
         <f t="array" ref="E1">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(F1 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!D$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!D$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Lecture Part 2</v>
+        <v>None</v>
       </c>
       <c r="F1" t="str" cm="1">
         <f t="array" ref="F1">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(G1 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!E$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!E$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="G1" t="str" cm="1">
         <f t="array" ref="G1">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(H1 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!F$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!F$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
@@ -2266,35 +1891,35 @@
       </c>
       <c r="K1" t="str" cm="1">
         <f t="array" ref="K1">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(L1 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!J$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!J$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Practical Part 1</v>
+        <v>None</v>
       </c>
       <c r="L1" t="str" cm="1">
         <f t="array" ref="L1">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!K$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(M1 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!K$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!K$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!K$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!K$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B4, " ", Timetable!K$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Practical Part 2</v>
+        <v>None</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
       </c>
       <c r="D2" t="str" cm="1">
         <f t="array" ref="D2">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(E2 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Practical Part 1</v>
+        <v>Lecture</v>
       </c>
       <c r="E2" t="str" cm="1">
         <f t="array" ref="E2">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(F2 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!D$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!D$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Practical Part 2</v>
+        <v>Lecture</v>
       </c>
       <c r="F2" t="str" cm="1">
         <f t="array" ref="F2">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(G2 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!E$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!E$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Practical Part 1</v>
+        <v>None</v>
       </c>
       <c r="G2" t="str" cm="1">
         <f t="array" ref="G2">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(H2 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!F$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!F$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Practical Part 2</v>
+        <v>None</v>
       </c>
       <c r="H2" t="str" cm="1">
         <f t="array" ref="H2">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(I2 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!G$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!G$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
@@ -2302,15 +1927,15 @@
       </c>
       <c r="I2" t="str" cm="1">
         <f t="array" ref="I2">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(J2 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!H$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!H$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="J2" t="str" cm="1">
         <f t="array" ref="J2">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(K2 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!I$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!I$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Practical Part 1</v>
+        <v>None</v>
       </c>
       <c r="K2" t="str" cm="1">
         <f t="array" ref="K2">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(L2 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!J$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!J$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Practical Part 2</v>
+        <v>None</v>
       </c>
       <c r="L2" t="str" cm="1">
         <f t="array" ref="L2">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!K$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(M2 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!K$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!K$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!K$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!K$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B5, " ", Timetable!K$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
@@ -2319,22 +1944,22 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
         <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
       </c>
       <c r="D3" t="str" cm="1">
         <f t="array" ref="D3">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(E3 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Workshop Part 1</v>
+        <v>None</v>
       </c>
       <c r="E3" t="str" cm="1">
         <f t="array" ref="E3">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(F3 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!D$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!D$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Workshop Part 2</v>
+        <v>None</v>
       </c>
       <c r="F3" t="str" cm="1">
         <f t="array" ref="F3">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(G3 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!E$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!E$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="G3" t="str" cm="1">
         <f t="array" ref="G3">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(H3 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!F$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B6, " ", Timetable!F$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
@@ -2363,18 +1988,18 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
       </c>
       <c r="D4" t="str" cm="1">
         <f t="array" ref="D4">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(E4 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Lecture</v>
+        <v>Lecture Part 1</v>
       </c>
       <c r="E4" t="str" cm="1">
         <f t="array" ref="E4">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(F4 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!D$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!D$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!D$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>None</v>
+        <v>Lecture Part 2</v>
       </c>
       <c r="F4" t="str" cm="1">
         <f t="array" ref="F4">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(G4 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!E$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!E$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!E$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
@@ -2386,11 +2011,11 @@
       </c>
       <c r="H4" t="str" cm="1">
         <f t="array" ref="H4">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(I4 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!G$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!G$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Lecture</v>
+        <v>None</v>
       </c>
       <c r="I4" t="str" cm="1">
         <f t="array" ref="I4">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(J4 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!H$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!H$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="J4" t="str" cm="1">
         <f t="array" ref="J4">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(K4 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!I$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B7, " ", Timetable!I$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
@@ -2407,10 +2032,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
         <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
       </c>
       <c r="D5" t="str" cm="1">
         <f t="array" ref="D5">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(E5 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!C$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!C$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
@@ -2426,7 +2051,7 @@
       </c>
       <c r="G5" t="str" cm="1">
         <f t="array" ref="G5">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(H5 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!F$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!F$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!F$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>Lecture</v>
+        <v>None</v>
       </c>
       <c r="H5" t="str" cm="1">
         <f t="array" ref="H5">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(I5 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!G$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!G$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!G$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
@@ -2434,11 +2059,11 @@
       </c>
       <c r="I5" t="str" cm="1">
         <f t="array" ref="I5">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(J5 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!H$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!H$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!H$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="J5" t="str" cm="1">
         <f t="array" ref="J5">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(K5 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!I$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!I$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!I$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
-        <v>None</v>
+        <v>Lecture</v>
       </c>
       <c r="K5" t="str" cm="1">
         <f t="array" ref="K5">_xlfn.IFS(_xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", IF(L5 = _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 1", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!J$3), Timetable!$J$28:$J$39, Timetable!$E$28:$E$39, " ", 0)), _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!J$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &lt;&gt; " ", _xlfn.XLOOKUP(_xlfn.CONCAT(Timetable!$B8, " ", Timetable!J$3), Timetable!$K$28:$K$39, Timetable!$E$28:$E$39, " ", 0) &amp; " Part 2", TRUE, "None")</f>
@@ -2451,10 +2076,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
         <v>21</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -2481,10 +2106,10 @@
         <v>2</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.35">
@@ -2504,18 +2129,18 @@
         <v>4</v>
       </c>
       <c r="H3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H4" t="s">
         <v>5</v>
@@ -2523,19 +2148,19 @@
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
       </c>
       <c r="D5" s="5">
         <v>0.5</v>
       </c>
       <c r="F5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H5" s="5">
         <v>0.5</v>
@@ -2543,13 +2168,13 @@
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" s="5">
         <v>0.25</v>
       </c>
       <c r="G6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H6" s="5">
         <v>0.25</v>
@@ -2557,13 +2182,13 @@
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" s="5">
         <v>0.25</v>
       </c>
       <c r="G7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H7" s="5">
         <v>0.25</v>
@@ -2571,16 +2196,16 @@
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="F9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.35">
@@ -2591,7 +2216,7 @@
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F10" t="s">
         <v>3</v>
@@ -2600,18 +2225,18 @@
         <v>4</v>
       </c>
       <c r="H10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
       </c>
       <c r="G11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H11" t="s">
         <v>5</v>
@@ -2619,19 +2244,19 @@
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
         <v>7</v>
-      </c>
-      <c r="C12" t="s">
-        <v>8</v>
       </c>
       <c r="D12" s="5">
         <v>0.5</v>
       </c>
       <c r="F12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G12" t="s">
         <v>7</v>
-      </c>
-      <c r="G12" t="s">
-        <v>8</v>
       </c>
       <c r="H12" s="5">
         <v>0.5</v>
@@ -2639,13 +2264,13 @@
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D13" s="5">
         <v>0.5</v>
       </c>
       <c r="G13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H13" s="5">
         <v>0.25</v>
@@ -2654,7 +2279,7 @@
     <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="D14" s="4"/>
       <c r="G14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H14" s="5">
         <v>0.25</v>
@@ -2662,16 +2287,16 @@
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="F16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.35">
@@ -2682,7 +2307,7 @@
         <v>4</v>
       </c>
       <c r="D17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F17" t="s">
         <v>3</v>
@@ -2691,18 +2316,18 @@
         <v>4</v>
       </c>
       <c r="H17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D18" t="s">
         <v>5</v>
       </c>
       <c r="G18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H18" t="s">
         <v>5</v>
@@ -2710,19 +2335,19 @@
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
         <v>7</v>
-      </c>
-      <c r="C19" t="s">
-        <v>8</v>
       </c>
       <c r="D19" s="5">
         <v>0.66</v>
       </c>
       <c r="F19" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H19" s="5">
         <v>0.05</v>
@@ -2730,14 +2355,14 @@
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D20" s="5">
         <f>0.33/2</f>
         <v>0.16500000000000001</v>
       </c>
       <c r="G20" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H20" s="5">
         <v>0.15</v>
@@ -2745,14 +2370,14 @@
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D21" s="5">
         <f>0.33/2</f>
         <v>0.16500000000000001</v>
       </c>
       <c r="G21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H21" s="5">
         <v>0.3</v>
@@ -2760,7 +2385,7 @@
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H22" s="5">
         <v>0.15</v>
@@ -2768,7 +2393,7 @@
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H23" s="5">
         <v>0.2</v>
@@ -2776,7 +2401,7 @@
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G24" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H24" s="5">
         <v>0.05</v>
@@ -2784,7 +2409,7 @@
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H25" s="5">
         <v>0.1</v>

</xml_diff>